<commit_message>
Correcion de modal y de planillas Alta y Act
</commit_message>
<xml_diff>
--- a/public/docs/planilla-vacia-actualizacionMasiva.xlsx
+++ b/public/docs/planilla-vacia-actualizacionMasiva.xlsx
@@ -5,22 +5,27 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\farme\OneDrive\Escritorio\WebNew\FARMERIN-Web-main-master-main-main-main\public\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\farme\OneDrive\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D224CC03-6DCE-46C2-83FA-21CF32A8A7E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3737AA4-C6B6-4D5B-993F-4A4DFD440237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>eRP (boton)</t>
   </si>
@@ -59,6 +64,9 @@
   </si>
   <si>
     <t>Fecha Servicio (dia/mes/año)</t>
+  </si>
+  <si>
+    <t>Grupo</t>
   </si>
 </sst>
 </file>
@@ -434,7 +442,9 @@
       <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="N1" s="5"/>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="O1" s="5"/>
       <c r="P1" s="5"/>
       <c r="Q1" s="5"/>
@@ -462,6 +472,7 @@
       <c r="K2" s="7"/>
       <c r="L2" s="8"/>
       <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A3" s="7"/>
@@ -477,6 +488,7 @@
       <c r="K3" s="7"/>
       <c r="L3" s="10"/>
       <c r="M3" s="7"/>
+      <c r="N3" s="7"/>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A4" s="7"/>
@@ -492,6 +504,7 @@
       <c r="K4" s="7"/>
       <c r="L4" s="10"/>
       <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A5" s="7"/>
@@ -507,6 +520,7 @@
       <c r="K5" s="7"/>
       <c r="L5" s="10"/>
       <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A6" s="7"/>
@@ -522,6 +536,7 @@
       <c r="K6" s="7"/>
       <c r="L6" s="10"/>
       <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A7" s="7"/>
@@ -537,6 +552,7 @@
       <c r="K7" s="7"/>
       <c r="L7" s="10"/>
       <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A8" s="7"/>
@@ -552,6 +568,7 @@
       <c r="K8" s="7"/>
       <c r="L8" s="10"/>
       <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
@@ -567,6 +584,7 @@
       <c r="K9" s="7"/>
       <c r="L9" s="10"/>
       <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A10" s="7"/>
@@ -582,6 +600,7 @@
       <c r="K10" s="7"/>
       <c r="L10" s="10"/>
       <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A11" s="7"/>
@@ -597,6 +616,7 @@
       <c r="K11" s="7"/>
       <c r="L11" s="10"/>
       <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A12" s="7"/>
@@ -612,6 +632,7 @@
       <c r="K12" s="7"/>
       <c r="L12" s="10"/>
       <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
@@ -627,6 +648,7 @@
       <c r="K13" s="7"/>
       <c r="L13" s="10"/>
       <c r="M13" s="7"/>
+      <c r="N13" s="7"/>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A14" s="7"/>
@@ -642,6 +664,7 @@
       <c r="K14" s="7"/>
       <c r="L14" s="10"/>
       <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
     </row>
     <row r="15" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A15" s="7"/>
@@ -657,6 +680,7 @@
       <c r="K15" s="7"/>
       <c r="L15" s="10"/>
       <c r="M15" s="7"/>
+      <c r="N15" s="7"/>
     </row>
     <row r="16" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A16" s="7"/>
@@ -672,8 +696,9 @@
       <c r="K16" s="7"/>
       <c r="L16" s="10"/>
       <c r="M16" s="7"/>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N16" s="7"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="7"/>
       <c r="B17" s="7"/>
       <c r="C17" s="10"/>
@@ -687,8 +712,9 @@
       <c r="K17" s="7"/>
       <c r="L17" s="10"/>
       <c r="M17" s="7"/>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N17" s="7"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="7"/>
       <c r="B18" s="7"/>
       <c r="C18" s="10"/>
@@ -702,8 +728,9 @@
       <c r="K18" s="7"/>
       <c r="L18" s="10"/>
       <c r="M18" s="7"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N18" s="7"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="7"/>
       <c r="B19" s="7"/>
       <c r="C19" s="10"/>
@@ -717,8 +744,9 @@
       <c r="K19" s="7"/>
       <c r="L19" s="10"/>
       <c r="M19" s="7"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N19" s="7"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="7"/>
       <c r="B20" s="7"/>
       <c r="C20" s="10"/>
@@ -732,8 +760,9 @@
       <c r="K20" s="7"/>
       <c r="L20" s="10"/>
       <c r="M20" s="7"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N20" s="7"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" s="7"/>
       <c r="B21" s="7"/>
       <c r="C21" s="10"/>
@@ -747,8 +776,9 @@
       <c r="K21" s="7"/>
       <c r="L21" s="10"/>
       <c r="M21" s="7"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N21" s="7"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" s="7"/>
       <c r="B22" s="7"/>
       <c r="C22" s="10"/>
@@ -762,8 +792,9 @@
       <c r="K22" s="7"/>
       <c r="L22" s="10"/>
       <c r="M22" s="7"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N22" s="7"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="7"/>
       <c r="B23" s="7"/>
       <c r="C23" s="10"/>
@@ -777,8 +808,9 @@
       <c r="K23" s="7"/>
       <c r="L23" s="10"/>
       <c r="M23" s="7"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N23" s="7"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="10"/>
@@ -792,8 +824,9 @@
       <c r="K24" s="7"/>
       <c r="L24" s="10"/>
       <c r="M24" s="7"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N24" s="7"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="10"/>
@@ -807,8 +840,9 @@
       <c r="K25" s="7"/>
       <c r="L25" s="10"/>
       <c r="M25" s="7"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N25" s="7"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="10"/>
@@ -822,8 +856,9 @@
       <c r="K26" s="7"/>
       <c r="L26" s="10"/>
       <c r="M26" s="7"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N26" s="7"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="7"/>
       <c r="B27" s="7"/>
       <c r="C27" s="10"/>
@@ -837,8 +872,9 @@
       <c r="K27" s="7"/>
       <c r="L27" s="10"/>
       <c r="M27" s="7"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N27" s="7"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="7"/>
       <c r="B28" s="7"/>
       <c r="C28" s="10"/>
@@ -852,8 +888,9 @@
       <c r="K28" s="7"/>
       <c r="L28" s="10"/>
       <c r="M28" s="7"/>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N28" s="7"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="7"/>
       <c r="B29" s="7"/>
       <c r="C29" s="10"/>
@@ -867,8 +904,9 @@
       <c r="K29" s="7"/>
       <c r="L29" s="10"/>
       <c r="M29" s="7"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N29" s="7"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="7"/>
       <c r="B30" s="7"/>
       <c r="C30" s="10"/>
@@ -882,8 +920,9 @@
       <c r="K30" s="7"/>
       <c r="L30" s="10"/>
       <c r="M30" s="7"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N30" s="7"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="7"/>
       <c r="B31" s="7"/>
       <c r="C31" s="10"/>
@@ -897,8 +936,9 @@
       <c r="K31" s="7"/>
       <c r="L31" s="10"/>
       <c r="M31" s="7"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N31" s="7"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="7"/>
       <c r="B32" s="7"/>
       <c r="C32" s="10"/>
@@ -912,8 +952,9 @@
       <c r="K32" s="7"/>
       <c r="L32" s="10"/>
       <c r="M32" s="7"/>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N32" s="7"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="7"/>
       <c r="B33" s="7"/>
       <c r="C33" s="10"/>
@@ -927,8 +968,9 @@
       <c r="K33" s="7"/>
       <c r="L33" s="10"/>
       <c r="M33" s="7"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N33" s="7"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="7"/>
       <c r="B34" s="7"/>
       <c r="C34" s="10"/>
@@ -942,8 +984,9 @@
       <c r="K34" s="7"/>
       <c r="L34" s="10"/>
       <c r="M34" s="7"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N34" s="7"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="7"/>
       <c r="B35" s="7"/>
       <c r="C35" s="10"/>
@@ -957,8 +1000,9 @@
       <c r="K35" s="7"/>
       <c r="L35" s="10"/>
       <c r="M35" s="7"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N35" s="7"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="7"/>
       <c r="B36" s="7"/>
       <c r="C36" s="10"/>
@@ -972,8 +1016,9 @@
       <c r="K36" s="7"/>
       <c r="L36" s="10"/>
       <c r="M36" s="7"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N36" s="7"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="7"/>
       <c r="B37" s="7"/>
       <c r="C37" s="10"/>
@@ -987,8 +1032,9 @@
       <c r="K37" s="7"/>
       <c r="L37" s="10"/>
       <c r="M37" s="7"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N37" s="7"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="7"/>
       <c r="B38" s="7"/>
       <c r="C38" s="10"/>
@@ -1002,8 +1048,9 @@
       <c r="K38" s="7"/>
       <c r="L38" s="10"/>
       <c r="M38" s="7"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N38" s="7"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="7"/>
       <c r="B39" s="7"/>
       <c r="C39" s="10"/>
@@ -1017,8 +1064,9 @@
       <c r="K39" s="7"/>
       <c r="L39" s="10"/>
       <c r="M39" s="7"/>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N39" s="7"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="7"/>
       <c r="B40" s="7"/>
       <c r="C40" s="10"/>
@@ -1032,8 +1080,9 @@
       <c r="K40" s="7"/>
       <c r="L40" s="10"/>
       <c r="M40" s="7"/>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N40" s="7"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="7"/>
       <c r="B41" s="7"/>
       <c r="C41" s="10"/>
@@ -1047,8 +1096,9 @@
       <c r="K41" s="7"/>
       <c r="L41" s="10"/>
       <c r="M41" s="7"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N41" s="7"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="7"/>
       <c r="B42" s="7"/>
       <c r="C42" s="10"/>
@@ -1062,8 +1112,9 @@
       <c r="K42" s="7"/>
       <c r="L42" s="10"/>
       <c r="M42" s="7"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N42" s="7"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
       <c r="C43" s="10"/>
@@ -1077,8 +1128,9 @@
       <c r="K43" s="7"/>
       <c r="L43" s="10"/>
       <c r="M43" s="7"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N43" s="7"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
       <c r="C44" s="10"/>
@@ -1092,8 +1144,9 @@
       <c r="K44" s="7"/>
       <c r="L44" s="10"/>
       <c r="M44" s="7"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N44" s="7"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="7"/>
       <c r="B45" s="7"/>
       <c r="C45" s="10"/>
@@ -1107,8 +1160,9 @@
       <c r="K45" s="7"/>
       <c r="L45" s="10"/>
       <c r="M45" s="7"/>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N45" s="7"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="7"/>
       <c r="B46" s="7"/>
       <c r="C46" s="10"/>
@@ -1122,8 +1176,9 @@
       <c r="K46" s="7"/>
       <c r="L46" s="10"/>
       <c r="M46" s="7"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N46" s="7"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="7"/>
       <c r="B47" s="7"/>
       <c r="C47" s="10"/>
@@ -1137,8 +1192,9 @@
       <c r="K47" s="7"/>
       <c r="L47" s="10"/>
       <c r="M47" s="7"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N47" s="7"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
       <c r="C48" s="10"/>
@@ -1152,8 +1208,9 @@
       <c r="K48" s="7"/>
       <c r="L48" s="10"/>
       <c r="M48" s="7"/>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N48" s="7"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="7"/>
       <c r="B49" s="7"/>
       <c r="C49" s="10"/>
@@ -1167,8 +1224,9 @@
       <c r="K49" s="7"/>
       <c r="L49" s="10"/>
       <c r="M49" s="7"/>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N49" s="7"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="7"/>
       <c r="B50" s="7"/>
       <c r="C50" s="10"/>
@@ -1182,86 +1240,87 @@
       <c r="K50" s="7"/>
       <c r="L50" s="10"/>
       <c r="M50" s="7"/>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="N50" s="7"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C51" s="11"/>
       <c r="G51" s="11"/>
       <c r="I51" s="12"/>
       <c r="L51" s="11"/>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C52" s="11"/>
       <c r="G52" s="11"/>
       <c r="I52" s="12"/>
       <c r="L52" s="11"/>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C53" s="11"/>
       <c r="G53" s="11"/>
       <c r="I53" s="12"/>
       <c r="L53" s="11"/>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C54" s="11"/>
       <c r="G54" s="11"/>
       <c r="I54" s="12"/>
       <c r="L54" s="11"/>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C55" s="11"/>
       <c r="G55" s="11"/>
       <c r="I55" s="12"/>
       <c r="L55" s="11"/>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C56" s="11"/>
       <c r="G56" s="11"/>
       <c r="I56" s="12"/>
       <c r="L56" s="11"/>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C57" s="11"/>
       <c r="G57" s="11"/>
       <c r="I57" s="12"/>
       <c r="L57" s="11"/>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C58" s="11"/>
       <c r="G58" s="11"/>
       <c r="I58" s="12"/>
       <c r="L58" s="11"/>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C59" s="11"/>
       <c r="G59" s="11"/>
       <c r="I59" s="12"/>
       <c r="L59" s="11"/>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C60" s="11"/>
       <c r="G60" s="11"/>
       <c r="I60" s="12"/>
       <c r="L60" s="11"/>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C61" s="11"/>
       <c r="G61" s="11"/>
       <c r="I61" s="12"/>
       <c r="L61" s="11"/>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C62" s="11"/>
       <c r="G62" s="11"/>
       <c r="I62" s="12"/>
       <c r="L62" s="11"/>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C63" s="11"/>
       <c r="G63" s="11"/>
       <c r="I63" s="12"/>
       <c r="L63" s="11"/>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="C64" s="11"/>
       <c r="G64" s="11"/>
       <c r="I64" s="12"/>

</xml_diff>